<commit_message>
Add new metrics to Excel benchmark plan
Add 7 metrics to the table: median, std dev, p95, p99 latency,
per-class accuracy, model file size, and GPU peak memory.
Update warm-up/measurement notes to mention CLI configurability.
</commit_message>
<xml_diff>
--- a/docs/plan_benchmark_yolo.xlsx
+++ b/docs/plan_benchmark_yolo.xlsx
@@ -588,7 +588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:M40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1589,7 +1589,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="29.15" customHeight="1">
       <c r="A18" s="1" t="inlineStr">
         <is>
@@ -1856,120 +1855,87 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Precisión</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>mAP50</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>Precisión media a IoU 0.50</t>
-        </is>
-      </c>
-      <c r="D24" s="17" t="n"/>
-      <c r="E24" s="18" t="n"/>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Velocidad</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Mediana</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Latencia mediana total (ms/img)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Precisión</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>mAP50-95</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>Precisión media promediada de IoU 0.50 a 0.95</t>
-        </is>
-      </c>
-      <c r="D25" s="17" t="n"/>
-      <c r="E25" s="18" t="n"/>
-      <c r="H25" s="13" t="inlineStr">
-        <is>
-          <t>Inferencia</t>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Velocidad</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Desv. estándar</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Desviación estándar de la latencia total (ms)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Precisión</t>
-        </is>
-      </c>
-      <c r="B26" s="15" t="inlineStr">
-        <is>
-          <t>Precision</t>
-        </is>
-      </c>
-      <c r="C26" s="16" t="inlineStr">
-        <is>
-          <t>Proporción de detecciones correctas sobre el total de detecciones realizadas por el modelo</t>
-        </is>
-      </c>
-      <c r="D26" s="17" t="n"/>
-      <c r="E26" s="18" t="n"/>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Warm-up </t>
-        </is>
-      </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>5 ejecuciones</t>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Velocidad</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>p95</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Percentil 95 de latencia total (ms/img)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Precisión</t>
-        </is>
-      </c>
-      <c r="B27" s="15" t="inlineStr">
-        <is>
-          <t>Recall</t>
-        </is>
-      </c>
-      <c r="C27" s="16" t="inlineStr">
-        <is>
-          <t>Proporción de objetos reales detectados correctamente sobre el total de objetos existentes</t>
-        </is>
-      </c>
-      <c r="D27" s="17" t="n"/>
-      <c r="E27" s="18" t="n"/>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>Mediciones</t>
-        </is>
-      </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>10 ejecuciones</t>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Velocidad</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>p99</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Percentil 99 de latencia total (ms/img)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>Eficiencia</t>
+          <t>Precisión</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Vatios</t>
+          <t>mAP50</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Consumo energético durante la inferencia (W)</t>
+          <t>Precisión media a IoU 0.50</t>
         </is>
       </c>
       <c r="D28" s="17" t="n"/>
@@ -1978,22 +1944,178 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>Eficiencia</t>
+          <t>Precisión</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>FPS/vatio</t>
+          <t>mAP50-95</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Eficiencia energética (solo Jetsons, vía jtop)</t>
+          <t>Precisión media promediada de IoU 0.50 a 0.95</t>
         </is>
       </c>
       <c r="D29" s="17" t="n"/>
       <c r="E29" s="18" t="n"/>
-    </row>
+      <c r="H29" s="13" t="inlineStr">
+        <is>
+          <t>Inferencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Precisión</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>Precision</t>
+        </is>
+      </c>
+      <c r="C30" s="16" t="inlineStr">
+        <is>
+          <t>Proporción de detecciones correctas sobre el total de detecciones realizadas por el modelo</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="n"/>
+      <c r="E30" s="18" t="n"/>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Warm-up </t>
+        </is>
+      </c>
+      <c r="I30" s="6" t="inlineStr">
+        <is>
+          <t>5 ejecuciones (configurable via --warmup)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Precisión</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>Recall</t>
+        </is>
+      </c>
+      <c r="C31" s="16" t="inlineStr">
+        <is>
+          <t>Proporción de objetos reales detectados correctamente sobre el total de objetos existentes</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="n"/>
+      <c r="E31" s="18" t="n"/>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>Mediciones</t>
+        </is>
+      </c>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>10 ejecuciones (configurable via --runs)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Precisión</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Métricas por clase</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>P, R, mAP50, mAP50-95 desglosados por cada una de las 8 clases</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Eficiencia</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Vatios</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>Consumo energético durante la inferencia (W)</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="n"/>
+      <c r="E33" s="18" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Eficiencia</t>
+        </is>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>FPS/vatio</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="inlineStr">
+        <is>
+          <t>Eficiencia energética (solo Jetsons, vía jtop)</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="n"/>
+      <c r="E34" s="18" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Recursos</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Tamaño del modelo</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Tamaño del archivo de pesos en disco (MB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Recursos</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Memoria GPU pico</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Memoria GPU máxima utilizada durante la inferencia (MB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="H25:I25"/>

</xml_diff>

<commit_message>
Add Experiment 5: class imbalance impact via weighted sampling
Implement weighted dataloader that samples images with probability
inversely proportional to their class frequency, addressing the 12x
imbalance between Solda (2,536) and IV-5 (218) in the weld dataset.

New files:
- scripts/weighted_sampler.py: computes per-image weights and
  monkey-patches Ultralytics build_dataloader

Changes:
- train.py: supports scratch_balanced/pretrained_balanced approaches
- experiments.yaml: Experiment 5 with all model sizes, both architectures
- infer.py: accepts balanced approach values
- docs: updated experiment design and run counts (376 inference, 520 total)
- Excel: added Experiment 5 rows and updated summary table
</commit_message>
<xml_diff>
--- a/docs/plan_benchmark_yolo.xlsx
+++ b/docs/plan_benchmark_yolo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tmp\TFM\ICM\BenchMarks\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05E77568-5898-4986-AD8D-A76B23AC9F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7690F29B-8F30-4A1B-974D-19F4028D9777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="92">
   <si>
     <t>Experimento</t>
   </si>
@@ -118,6 +118,18 @@
     <t>Detección</t>
   </si>
   <si>
+    <t>Desequilibrio clases</t>
+  </si>
+  <si>
+    <t>Desde cero (balanceado)</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>Transfer learning (balanceado)</t>
+  </si>
+  <si>
     <t>Categoría</t>
   </si>
   <si>
@@ -183,6 +195,9 @@
     <t>Suma de las tres anteriores (ms/img)</t>
   </si>
   <si>
+    <t>Desequilibrio</t>
+  </si>
+  <si>
     <t>FPS</t>
   </si>
   <si>
@@ -210,12 +225,24 @@
     <t>Percentil 95 de latencia total (ms/img)</t>
   </si>
   <si>
+    <t xml:space="preserve">Warm-up </t>
+  </si>
+  <si>
+    <t>5 ejecuciones (configurable via --warmup)</t>
+  </si>
+  <si>
     <t>p99</t>
   </si>
   <si>
     <t>Percentil 99 de latencia total (ms/img)</t>
   </si>
   <si>
+    <t>Mediciones</t>
+  </si>
+  <si>
+    <t>10 ejecuciones (configurable via --runs)</t>
+  </si>
+  <si>
     <t>Precisión</t>
   </si>
   <si>
@@ -237,22 +264,10 @@
     <t>Proporción de detecciones correctas sobre el total de detecciones realizadas por el modelo</t>
   </si>
   <si>
-    <t xml:space="preserve">Warm-up </t>
-  </si>
-  <si>
-    <t>5 ejecuciones (configurable via --warmup)</t>
-  </si>
-  <si>
     <t>Recall</t>
   </si>
   <si>
     <t>Proporción de objetos reales detectados correctamente sobre el total de objetos existentes</t>
-  </si>
-  <si>
-    <t>Mediciones</t>
-  </si>
-  <si>
-    <t>10 ejecuciones (configurable via --runs)</t>
   </si>
   <si>
     <t>Métricas por clase</t>
@@ -332,7 +347,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -366,6 +381,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE4EC"/>
+        <bgColor rgb="FFFCE4EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor rgb="FFFCE4EC"/>
       </patternFill>
     </fill>
@@ -443,7 +464,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -478,28 +499,31 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -804,7 +828,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1476,419 +1500,528 @@
         <v>21</v>
       </c>
     </row>
+    <row r="17" spans="1:13" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="12">
+        <v>5</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" s="12">
+        <v>640</v>
+      </c>
+      <c r="G17" s="12">
+        <v>1</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="I17" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="J17" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="K17" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="L17" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="M17" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
     <row r="18" spans="1:13" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="12">
+        <v>5</v>
+      </c>
+      <c r="B18" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" s="12">
+        <v>640</v>
+      </c>
+      <c r="G18" s="12">
+        <v>1</v>
+      </c>
+      <c r="H18" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="I18" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="J18" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="K18" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="L18" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="G18" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="I18" s="8" t="s">
+      <c r="M18" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="16"/>
+    </row>
+    <row r="20" spans="1:13" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="J18" s="8" t="s">
+      <c r="B20" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="K18" s="8" t="s">
+      <c r="C20" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="L18" s="8" t="s">
+      <c r="D20" s="16"/>
+      <c r="E20" s="16"/>
+      <c r="G20" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="M18" s="8" t="s">
+      <c r="H20" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="I20" s="8" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A19" s="6" t="s">
+      <c r="J20" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="K20" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="L20" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D19" s="14"/>
-      <c r="E19" s="15"/>
-      <c r="G19" s="2">
-        <v>1</v>
-      </c>
-      <c r="H19" s="2" t="s">
+      <c r="M20" s="8" t="s">
         <v>43</v>
-      </c>
-      <c r="I19" s="2">
-        <v>16</v>
-      </c>
-      <c r="J19" s="2">
-        <v>48</v>
-      </c>
-      <c r="K19" s="2">
-        <v>48</v>
-      </c>
-      <c r="L19" s="2">
-        <v>48</v>
-      </c>
-      <c r="M19" s="2">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A20" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="D20" s="14"/>
-      <c r="E20" s="15"/>
-      <c r="G20" s="3">
-        <v>2</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="I20" s="3">
-        <v>0</v>
-      </c>
-      <c r="J20" s="3">
-        <v>32</v>
-      </c>
-      <c r="K20" s="3">
-        <v>32</v>
-      </c>
-      <c r="L20" s="3">
-        <v>32</v>
-      </c>
-      <c r="M20" s="3">
-        <v>96</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A21" s="6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B21" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="13" t="s">
         <v>46</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>47</v>
       </c>
       <c r="D21" s="14"/>
       <c r="E21" s="15"/>
-      <c r="G21" s="4">
-        <v>3</v>
-      </c>
-      <c r="H21" s="4" t="s">
+      <c r="G21" s="2">
+        <v>1</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I21" s="2">
+        <v>16</v>
+      </c>
+      <c r="J21" s="2">
         <v>48</v>
       </c>
-      <c r="I21" s="4">
-        <v>0</v>
-      </c>
-      <c r="J21" s="4">
-        <v>24</v>
-      </c>
-      <c r="K21" s="4">
-        <v>24</v>
-      </c>
-      <c r="L21" s="4">
-        <v>24</v>
-      </c>
-      <c r="M21" s="4">
-        <v>72</v>
+      <c r="K21" s="2">
+        <v>48</v>
+      </c>
+      <c r="L21" s="2">
+        <v>48</v>
+      </c>
+      <c r="M21" s="2">
+        <v>144</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A22" s="6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D22" s="14"/>
       <c r="E22" s="15"/>
-      <c r="G22" s="5">
-        <v>4</v>
-      </c>
-      <c r="H22" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="I22" s="5">
-        <v>16</v>
-      </c>
-      <c r="J22" s="5">
-        <v>16</v>
-      </c>
-      <c r="K22" s="5">
-        <v>16</v>
-      </c>
-      <c r="L22" s="5">
-        <v>16</v>
-      </c>
-      <c r="M22" s="5">
-        <v>48</v>
+      <c r="G22" s="3">
+        <v>2</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="I22" s="3">
+        <v>0</v>
+      </c>
+      <c r="J22" s="3">
+        <v>32</v>
+      </c>
+      <c r="K22" s="3">
+        <v>32</v>
+      </c>
+      <c r="L22" s="3">
+        <v>32</v>
+      </c>
+      <c r="M22" s="3">
+        <v>96</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A23" s="6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B23" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" s="13" t="s">
         <v>51</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>52</v>
       </c>
       <c r="D23" s="14"/>
       <c r="E23" s="15"/>
-      <c r="G23" s="9"/>
-      <c r="H23" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="I23" s="9">
-        <v>32</v>
-      </c>
-      <c r="J23" s="9">
-        <v>120</v>
-      </c>
-      <c r="K23" s="9">
-        <v>120</v>
-      </c>
-      <c r="L23" s="9">
-        <v>120</v>
-      </c>
-      <c r="M23" s="9">
-        <v>360</v>
+      <c r="G23" s="4">
+        <v>3</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="I23" s="4">
+        <v>0</v>
+      </c>
+      <c r="J23" s="4">
+        <v>24</v>
+      </c>
+      <c r="K23" s="4">
+        <v>24</v>
+      </c>
+      <c r="L23" s="4">
+        <v>24</v>
+      </c>
+      <c r="M23" s="4">
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A24" s="6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B24" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C24" s="13" t="s">
         <v>54</v>
-      </c>
-      <c r="C24" s="13" t="s">
-        <v>55</v>
       </c>
       <c r="D24" s="14"/>
       <c r="E24" s="15"/>
+      <c r="G24" s="5">
+        <v>4</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="I24" s="5">
+        <v>16</v>
+      </c>
+      <c r="J24" s="5">
+        <v>16</v>
+      </c>
+      <c r="K24" s="5">
+        <v>16</v>
+      </c>
+      <c r="L24" s="5">
+        <v>16</v>
+      </c>
+      <c r="M24" s="5">
+        <v>48</v>
+      </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A25" s="6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="13" t="s">
+      <c r="C25" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="D25" s="14"/>
-      <c r="E25" s="15"/>
-      <c r="H25" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="D25" s="21"/>
+      <c r="E25" s="22"/>
+      <c r="G25" s="12">
+        <v>5</v>
+      </c>
+      <c r="H25" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="I25" s="12">
+        <v>16</v>
+      </c>
+      <c r="J25" s="12">
+        <v>16</v>
+      </c>
+      <c r="K25" s="12">
+        <v>0</v>
+      </c>
+      <c r="L25" s="12">
+        <v>0</v>
+      </c>
+      <c r="M25" s="12">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A26" s="6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B26" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="D26" s="21"/>
+      <c r="E26" s="22"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="C26" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="D26" s="14"/>
-      <c r="E26" s="15"/>
-      <c r="H26" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="I26" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="J26" s="21"/>
-      <c r="K26" s="21"/>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="I26" s="9">
+        <v>48</v>
+      </c>
+      <c r="J26" s="9">
+        <v>136</v>
+      </c>
+      <c r="K26" s="9">
+        <v>120</v>
+      </c>
+      <c r="L26" s="9">
+        <v>120</v>
+      </c>
+      <c r="M26" s="9">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A27" s="6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="C27" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="D27" s="14"/>
-      <c r="E27" s="15"/>
-      <c r="H27" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="I27" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="J27" s="21"/>
-      <c r="K27" s="21"/>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="C27" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="D27" s="21"/>
+      <c r="E27" s="22"/>
+    </row>
+    <row r="28" spans="1:13" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A28" s="6" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="13" t="s">
+      <c r="C28" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="D28" s="14"/>
-      <c r="E28" s="15"/>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="D28" s="21"/>
+      <c r="E28" s="22"/>
+      <c r="H28" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A29" s="6" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="B29" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="D29" s="21"/>
+      <c r="E29" s="22"/>
+      <c r="H29" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="C29" s="13" t="s">
+      <c r="I29" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="D29" s="14"/>
-      <c r="E29" s="15"/>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="J29" s="19"/>
+      <c r="K29" s="19"/>
+    </row>
+    <row r="30" spans="1:13" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A30" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="B30" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="C30" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="D30" s="18"/>
-      <c r="E30" s="19"/>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.4">
+        <v>71</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="D30" s="21"/>
+      <c r="E30" s="22"/>
+      <c r="H30" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="I30" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="J30" s="19"/>
+      <c r="K30" s="19"/>
+    </row>
+    <row r="31" spans="1:13" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A31" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="B31" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="C31" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="D31" s="18"/>
-      <c r="E31" s="19"/>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="B31" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="D31" s="21"/>
+      <c r="E31" s="22"/>
+    </row>
+    <row r="32" spans="1:13" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A32" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="C32" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="B32" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="D32" s="14"/>
-      <c r="E32" s="15"/>
+      <c r="C32" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="D32" s="21"/>
+      <c r="E32" s="22"/>
     </row>
     <row r="33" spans="1:5" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="B33" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B33" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="C33" s="13" t="s">
+      <c r="C33" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="D33" s="14"/>
-      <c r="E33" s="15"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="22"/>
     </row>
     <row r="34" spans="1:5" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="6" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B34" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C34" s="13" t="s">
+      <c r="C34" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="D34" s="14"/>
-      <c r="E34" s="15"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="D34" s="21"/>
+      <c r="E34" s="22"/>
+    </row>
+    <row r="35" spans="1:5" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" s="6" t="s">
         <v>82</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="C35" s="13" t="s">
+      <c r="C35" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="D35" s="14"/>
-      <c r="E35" s="15"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="D35" s="21"/>
+      <c r="E35" s="22"/>
+    </row>
+    <row r="36" spans="1:5" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="6" t="s">
         <v>82</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="C36" s="13" t="s">
+      <c r="C36" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="D36" s="14"/>
-      <c r="E36" s="15"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="22"/>
+    </row>
+    <row r="37" spans="1:5" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A37" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C37" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="D37" s="21"/>
+      <c r="E37" s="22"/>
+    </row>
+    <row r="38" spans="1:5" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A38" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C38" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38" s="21"/>
+      <c r="E38" s="22"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="C34:E34"/>
+  <mergeCells count="22">
+    <mergeCell ref="C38:E38"/>
     <mergeCell ref="C32:E32"/>
-    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="I29:K29"/>
+    <mergeCell ref="I30:K30"/>
+    <mergeCell ref="C37:E37"/>
     <mergeCell ref="C36:E36"/>
-    <mergeCell ref="C30:E30"/>
-    <mergeCell ref="I26:K26"/>
-    <mergeCell ref="I27:K27"/>
-    <mergeCell ref="C31:E31"/>
     <mergeCell ref="C33:E33"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="C26:E26"/>
-    <mergeCell ref="C29:E29"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C25:E25"/>
-    <mergeCell ref="C24:E24"/>
     <mergeCell ref="C28:E28"/>
     <mergeCell ref="C27:E27"/>
     <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C34:E34"/>
+    <mergeCell ref="C31:E31"/>
     <mergeCell ref="C23:E23"/>
     <mergeCell ref="C22:E22"/>
+    <mergeCell ref="C26:E26"/>
+    <mergeCell ref="C29:E29"/>
+    <mergeCell ref="C30:E30"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C35:E35"/>
+    <mergeCell ref="C25:E25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Switch training batch to AutoBatch and update Excel plan
Change batch from fixed 16 to -1 (AutoBatch) so each model uses
the largest batch that fits in GPU memory. The benchmark aims to
find the best real-world configuration, not compare under identical
artificial constraints.

Excel updated with new columns (Dataset, Batch Entren., Batch Inf.)
reflecting the balanced/unbalanced and AutoBatch design.
</commit_message>
<xml_diff>
--- a/docs/plan_benchmark_yolo.xlsx
+++ b/docs/plan_benchmark_yolo.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tmp\TFM\ICM\BenchMarks\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7690F29B-8F30-4A1B-974D-19F4028D9777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65CF7EBC-0DEA-45E9-B7B2-324FCDEDFBC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Diseño experimental" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="95">
   <si>
     <t>Experimento</t>
   </si>
@@ -41,9 +54,6 @@
     <t>Entrada</t>
   </si>
   <si>
-    <t>Batch</t>
-  </si>
-  <si>
     <t>Arquitectura
 YoLo</t>
   </si>
@@ -121,13 +131,7 @@
     <t>Desequilibrio clases</t>
   </si>
   <si>
-    <t>Desde cero (balanceado)</t>
-  </si>
-  <si>
     <t>—</t>
-  </si>
-  <si>
-    <t>Transfer learning (balanceado)</t>
   </si>
   <si>
     <t>Categoría</t>
@@ -304,6 +308,26 @@
   </si>
   <si>
     <t>Memoria GPU máxima utilizada durante la inferencia (MB)</t>
+  </si>
+  <si>
+    <t>Batch
+Entren.</t>
+  </si>
+  <si>
+    <t>Batch
+Inf.</t>
+  </si>
+  <si>
+    <t>Dataset</t>
+  </si>
+  <si>
+    <t>Balanceado</t>
+  </si>
+  <si>
+    <t>Desbalanceado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AutoBatch </t>
   </si>
 </sst>
 </file>
@@ -464,7 +488,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -502,6 +526,15 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -509,21 +542,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -828,7 +846,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:O38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -837,14 +855,16 @@
     <col min="4" max="4" width="18" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="9" customWidth="1"/>
-    <col min="7" max="7" width="7" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="7" max="7" width="13.84375" customWidth="1"/>
+    <col min="8" max="8" width="10.921875" customWidth="1"/>
+    <col min="9" max="9" width="7" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="11" max="13" width="16" customWidth="1"/>
+    <col min="11" max="11" width="15" customWidth="1"/>
+    <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="13" max="15" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:15" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -864,1152 +884,1250 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="N1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="O1" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="8" t="s">
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A2" s="2">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>16</v>
       </c>
       <c r="F2" s="2">
         <v>640</v>
       </c>
-      <c r="G2" s="2">
-        <v>1</v>
+      <c r="G2" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="H2" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I2" s="2">
+        <v>1</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="L2" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="7" t="s">
+      <c r="M2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="L2" s="2" t="s">
+      <c r="N2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="M2" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A3" s="2">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="F3" s="2">
         <v>640</v>
       </c>
-      <c r="G3" s="2">
-        <v>1</v>
+      <c r="G3" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="H3" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I3" s="2">
+        <v>1</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="L3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="M3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="N3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>16</v>
       </c>
       <c r="F4" s="2">
         <v>640</v>
       </c>
-      <c r="G4" s="2">
-        <v>1</v>
+      <c r="G4" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="H4" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I4" s="2">
+        <v>1</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="M4" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.4">
+        <v>24</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>1</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="F5" s="2">
         <v>640</v>
       </c>
-      <c r="G5" s="2">
-        <v>1</v>
+      <c r="G5" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="H5" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I5" s="2">
+        <v>1</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="L5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K5" s="2" t="s">
+      <c r="M5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A6" s="2">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="L5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A6" s="2">
-        <v>1</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="D6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>15</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>16</v>
       </c>
       <c r="F6" s="2">
         <v>640</v>
       </c>
-      <c r="G6" s="2">
-        <v>1</v>
+      <c r="G6" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="H6" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I6" s="2">
+        <v>1</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="L6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K6" s="2" t="s">
+      <c r="M6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A7" s="2">
+        <v>1</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="L6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A7" s="2">
-        <v>1</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>26</v>
-      </c>
       <c r="D7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="F7" s="2">
         <v>640</v>
       </c>
-      <c r="G7" s="2">
-        <v>1</v>
+      <c r="G7" s="2" t="s">
+        <v>93</v>
       </c>
       <c r="H7" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="I7" s="2">
+        <v>1</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="K7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="L7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="J7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="M7" s="2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.4">
+        <v>24</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A8" s="3">
         <v>2</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>16</v>
       </c>
       <c r="F8" s="3">
         <v>320</v>
       </c>
-      <c r="G8" s="3">
-        <v>1</v>
+      <c r="G8" s="3" t="s">
+        <v>93</v>
       </c>
       <c r="H8" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="I8" s="3">
+        <v>1</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="L8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J8" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>21</v>
-      </c>
       <c r="M8" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="N8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="O8" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A9" s="3">
         <v>2</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="F9" s="3">
         <v>320</v>
       </c>
-      <c r="G9" s="3">
-        <v>1</v>
+      <c r="G9" s="3" t="s">
+        <v>93</v>
       </c>
       <c r="H9" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="I9" s="3">
+        <v>1</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K9" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="3" t="s">
+      <c r="L9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J9" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>21</v>
-      </c>
       <c r="M9" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="N9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="O9" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A10" s="3">
         <v>2</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>16</v>
       </c>
       <c r="F10" s="3">
         <v>1280</v>
       </c>
-      <c r="G10" s="3">
-        <v>1</v>
+      <c r="G10" s="3" t="s">
+        <v>93</v>
       </c>
       <c r="H10" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="I10" s="3">
+        <v>1</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="L10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J10" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>21</v>
-      </c>
       <c r="M10" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="N10" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="O10" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A11" s="3">
         <v>2</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D11" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="F11" s="3">
         <v>1280</v>
       </c>
-      <c r="G11" s="3">
-        <v>1</v>
+      <c r="G11" s="3" t="s">
+        <v>93</v>
       </c>
       <c r="H11" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="I11" s="3">
+        <v>1</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K11" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="I11" s="3" t="s">
+      <c r="L11" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="J11" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>21</v>
-      </c>
       <c r="M11" s="3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="O11" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A12" s="4">
         <v>3</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C12" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>16</v>
       </c>
       <c r="F12" s="4">
         <v>640</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="I12" s="4">
         <v>4</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="J12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="L12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J12" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L12" s="4" t="s">
-        <v>21</v>
-      </c>
       <c r="M12" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="N12" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="O12" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A13" s="4">
         <v>3</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>16</v>
       </c>
       <c r="F13" s="4">
         <v>640</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="I13" s="4">
         <v>8</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="J13" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K13" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="L13" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J13" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K13" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L13" s="4" t="s">
-        <v>21</v>
-      </c>
       <c r="M13" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="N13" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="O13" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A14" s="4">
         <v>3</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C14" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>16</v>
       </c>
       <c r="F14" s="4">
         <v>640</v>
       </c>
-      <c r="G14" s="4">
-        <v>16</v>
+      <c r="G14" s="4" t="s">
+        <v>93</v>
       </c>
       <c r="H14" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="I14" s="4">
+        <v>16</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="K14" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="L14" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="J14" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L14" s="4" t="s">
-        <v>21</v>
-      </c>
       <c r="M14" s="4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.4">
+        <v>20</v>
+      </c>
+      <c r="N14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="O14" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A15" s="5">
         <v>4</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C15" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="5" t="s">
         <v>15</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>16</v>
       </c>
       <c r="F15" s="5">
         <v>640</v>
       </c>
-      <c r="G15" s="5">
-        <v>1</v>
+      <c r="G15" s="5" t="s">
+        <v>93</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>30</v>
+        <v>94</v>
+      </c>
+      <c r="I15" s="5">
+        <v>1</v>
       </c>
       <c r="J15" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L15" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="M15" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="K15" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="L15" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="M15" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="N15" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="O15" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A16" s="5">
         <v>4</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D16" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="5" t="s">
         <v>22</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>23</v>
       </c>
       <c r="F16" s="5">
         <v>640</v>
       </c>
-      <c r="G16" s="5">
-        <v>1</v>
+      <c r="G16" s="5" t="s">
+        <v>93</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="I16" s="5" t="s">
-        <v>30</v>
+        <v>94</v>
+      </c>
+      <c r="I16" s="5">
+        <v>1</v>
       </c>
       <c r="J16" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="L16" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="M16" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="K16" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="L16" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="M16" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="N16" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="O16" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A17" s="12">
         <v>5</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C17" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="12" t="s">
-        <v>32</v>
-      </c>
       <c r="E17" s="12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F17" s="12">
         <v>640</v>
       </c>
-      <c r="G17" s="12">
-        <v>1</v>
+      <c r="G17" s="12" t="s">
+        <v>92</v>
       </c>
       <c r="H17" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="I17" s="12">
+        <v>1</v>
+      </c>
+      <c r="J17" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="K17" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="I17" s="12" t="s">
+      <c r="L17" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="J17" s="12" t="s">
+      <c r="M17" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="K17" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="L17" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="M17" s="12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="N17" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="O17" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A18" s="12">
         <v>5</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F18" s="12">
         <v>640</v>
       </c>
-      <c r="G18" s="12">
-        <v>1</v>
+      <c r="G18" s="12" t="s">
+        <v>92</v>
       </c>
       <c r="H18" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="I18" s="12">
+        <v>1</v>
+      </c>
+      <c r="J18" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="K18" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="I18" s="12" t="s">
+      <c r="L18" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="J18" s="12" t="s">
+      <c r="M18" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="K18" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="L18" s="12" t="s">
+      <c r="N18" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="O18" s="12" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+    </row>
+    <row r="20" spans="1:15" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A20" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="M18" s="12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="C19" s="16"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
-    </row>
-    <row r="20" spans="1:13" ht="29.15" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="1" t="s">
+      <c r="C20" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19"/>
+      <c r="I20" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="J20" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="K20" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="L20" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="G20" s="8" t="s">
+      <c r="M20" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="H20" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="I20" s="8" t="s">
+      <c r="N20" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="J20" s="8" t="s">
+      <c r="O20" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="K20" s="8" t="s">
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A21" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="L20" s="8" t="s">
+      <c r="B21" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="M20" s="8" t="s">
+      <c r="C21" s="16" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A21" s="6" t="s">
+      <c r="D21" s="17"/>
+      <c r="E21" s="18"/>
+      <c r="I21" s="2">
+        <v>1</v>
+      </c>
+      <c r="J21" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="D21" s="14"/>
-      <c r="E21" s="15"/>
-      <c r="G21" s="2">
-        <v>1</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="I21" s="2">
-        <v>16</v>
-      </c>
-      <c r="J21" s="2">
-        <v>48</v>
-      </c>
       <c r="K21" s="2">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="L21" s="2">
         <v>48</v>
       </c>
       <c r="M21" s="2">
+        <v>48</v>
+      </c>
+      <c r="N21" s="2">
+        <v>48</v>
+      </c>
+      <c r="O21" s="2">
         <v>144</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A22" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="D22" s="14"/>
-      <c r="E22" s="15"/>
-      <c r="G22" s="3">
+        <v>20</v>
+      </c>
+      <c r="C22" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="D22" s="17"/>
+      <c r="E22" s="18"/>
+      <c r="I22" s="3">
         <v>2</v>
       </c>
-      <c r="H22" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="I22" s="3">
+      <c r="J22" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="K22" s="3">
         <v>0</v>
-      </c>
-      <c r="J22" s="3">
-        <v>32</v>
-      </c>
-      <c r="K22" s="3">
-        <v>32</v>
       </c>
       <c r="L22" s="3">
         <v>32</v>
       </c>
       <c r="M22" s="3">
+        <v>32</v>
+      </c>
+      <c r="N22" s="3">
+        <v>32</v>
+      </c>
+      <c r="O22" s="3">
         <v>96</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A23" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="D23" s="14"/>
-      <c r="E23" s="15"/>
-      <c r="G23" s="4">
+        <v>47</v>
+      </c>
+      <c r="C23" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" s="17"/>
+      <c r="E23" s="18"/>
+      <c r="I23" s="4">
         <v>3</v>
       </c>
-      <c r="H23" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="I23" s="4">
+      <c r="J23" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="K23" s="4">
         <v>0</v>
-      </c>
-      <c r="J23" s="4">
-        <v>24</v>
-      </c>
-      <c r="K23" s="4">
-        <v>24</v>
       </c>
       <c r="L23" s="4">
         <v>24</v>
       </c>
       <c r="M23" s="4">
+        <v>24</v>
+      </c>
+      <c r="N23" s="4">
+        <v>24</v>
+      </c>
+      <c r="O23" s="4">
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.4">
       <c r="A24" s="6" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B24" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" s="17"/>
+      <c r="E24" s="18"/>
+      <c r="I24" s="5">
+        <v>4</v>
+      </c>
+      <c r="J24" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="K24" s="5">
+        <v>16</v>
+      </c>
+      <c r="L24" s="5">
+        <v>16</v>
+      </c>
+      <c r="M24" s="5">
+        <v>16</v>
+      </c>
+      <c r="N24" s="5">
+        <v>16</v>
+      </c>
+      <c r="O24" s="5">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.4">
+      <c r="A25" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C24" s="13" t="s">
+      <c r="C25" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="D24" s="14"/>
-      <c r="E24" s="15"/>
-      <c r="G24" s="5">
-        <v>4</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="I24" s="5">
-        <v>16</v>
-      </c>
-      <c r="J24" s="5">
-        <v>16</v>
-      </c>
-      <c r="K24" s="5">
-        <v>16</v>
-      </c>
-      <c r="L24" s="5">
-        <v>16</v>
-      </c>
-      <c r="M24" s="5">
+      <c r="D25" s="14"/>
+      <c r="E25" s="15"/>
+      <c r="I25" s="12">
+        <v>5</v>
+      </c>
+      <c r="J25" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="K25" s="12">
+        <v>16</v>
+      </c>
+      <c r="L25" s="12">
+        <v>16</v>
+      </c>
+      <c r="M25" s="12">
+        <v>0</v>
+      </c>
+      <c r="N25" s="12">
+        <v>0</v>
+      </c>
+      <c r="O25" s="12">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A26" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D26" s="14"/>
+      <c r="E26" s="15"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="K26" s="9">
         <v>48</v>
       </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A25" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C25" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="D25" s="21"/>
-      <c r="E25" s="22"/>
-      <c r="G25" s="12">
-        <v>5</v>
-      </c>
-      <c r="H25" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="I25" s="12">
-        <v>16</v>
-      </c>
-      <c r="J25" s="12">
-        <v>16</v>
-      </c>
-      <c r="K25" s="12">
-        <v>0</v>
-      </c>
-      <c r="L25" s="12">
-        <v>0</v>
-      </c>
-      <c r="M25" s="12">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B26" s="6" t="s">
+      <c r="L26" s="9">
+        <v>136</v>
+      </c>
+      <c r="M26" s="9">
+        <v>120</v>
+      </c>
+      <c r="N26" s="9">
+        <v>120</v>
+      </c>
+      <c r="O26" s="9">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="C27" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="C26" s="20" t="s">
+      <c r="D27" s="14"/>
+      <c r="E27" s="15"/>
+    </row>
+    <row r="28" spans="1:15" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A28" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="D26" s="21"/>
-      <c r="E26" s="22"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="I26" s="9">
-        <v>48</v>
-      </c>
-      <c r="J26" s="9">
-        <v>136</v>
-      </c>
-      <c r="K26" s="9">
-        <v>120</v>
-      </c>
-      <c r="L26" s="9">
-        <v>120</v>
-      </c>
-      <c r="M26" s="9">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A27" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B27" s="6" t="s">
+      <c r="C28" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="20" t="s">
+      <c r="D28" s="14"/>
+      <c r="E28" s="15"/>
+      <c r="J28" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A29" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="D29" s="14"/>
+      <c r="E29" s="15"/>
+      <c r="J29" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D27" s="21"/>
-      <c r="E27" s="22"/>
-    </row>
-    <row r="28" spans="1:13" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A28" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B28" s="6" t="s">
+      <c r="K29" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C28" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="D28" s="21"/>
-      <c r="E28" s="22"/>
-      <c r="H28" s="10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B29" s="6" t="s">
+      <c r="L29" s="14"/>
+      <c r="M29" s="15"/>
+    </row>
+    <row r="30" spans="1:15" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A30" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="D30" s="14"/>
+      <c r="E30" s="15"/>
+      <c r="J30" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="K30" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="C29" s="20" t="s">
+      <c r="L30" s="14"/>
+      <c r="M30" s="15"/>
+    </row>
+    <row r="31" spans="1:15" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A31" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="D29" s="21"/>
-      <c r="E29" s="22"/>
-      <c r="H29" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="I29" s="18" t="s">
-        <v>66</v>
-      </c>
-      <c r="J29" s="19"/>
-      <c r="K29" s="19"/>
-    </row>
-    <row r="30" spans="1:13" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="6" t="s">
+      <c r="B31" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="C31" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="C30" s="20" t="s">
+      <c r="D31" s="14"/>
+      <c r="E31" s="15"/>
+    </row>
+    <row r="32" spans="1:15" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="A32" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B32" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D30" s="21"/>
-      <c r="E30" s="22"/>
-      <c r="H30" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="I30" s="18" t="s">
-        <v>70</v>
-      </c>
-      <c r="J30" s="19"/>
-      <c r="K30" s="19"/>
-    </row>
-    <row r="31" spans="1:13" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B31" s="6" t="s">
+      <c r="C32" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="C31" s="20" t="s">
-        <v>75</v>
-      </c>
-      <c r="D31" s="21"/>
-      <c r="E31" s="22"/>
-    </row>
-    <row r="32" spans="1:13" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="C32" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="D32" s="21"/>
-      <c r="E32" s="22"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="15"/>
     </row>
     <row r="33" spans="1:5" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A33" s="6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="C33" s="20" t="s">
-        <v>79</v>
-      </c>
-      <c r="D33" s="21"/>
-      <c r="E33" s="22"/>
+        <v>75</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="D33" s="14"/>
+      <c r="E33" s="15"/>
     </row>
     <row r="34" spans="1:5" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A34" s="6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C34" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="D34" s="21"/>
-      <c r="E34" s="22"/>
+        <v>77</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="D34" s="14"/>
+      <c r="E34" s="15"/>
     </row>
     <row r="35" spans="1:5" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A35" s="6" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="C35" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="D35" s="21"/>
-      <c r="E35" s="22"/>
+        <v>80</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="D35" s="14"/>
+      <c r="E35" s="15"/>
     </row>
     <row r="36" spans="1:5" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A36" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B36" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="B36" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="C36" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="D36" s="21"/>
-      <c r="E36" s="22"/>
+      <c r="C36" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="D36" s="14"/>
+      <c r="E36" s="15"/>
     </row>
     <row r="37" spans="1:5" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A37" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="C37" s="20" t="s">
-        <v>89</v>
-      </c>
-      <c r="D37" s="21"/>
-      <c r="E37" s="22"/>
+        <v>85</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D37" s="14"/>
+      <c r="E37" s="15"/>
     </row>
     <row r="38" spans="1:5" ht="14.6" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A38" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B38" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B38" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="C38" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="D38" s="21"/>
-      <c r="E38" s="22"/>
+      <c r="C38" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D38" s="14"/>
+      <c r="E38" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="C38:E38"/>
-    <mergeCell ref="C32:E32"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="I29:K29"/>
-    <mergeCell ref="I30:K30"/>
-    <mergeCell ref="C37:E37"/>
-    <mergeCell ref="C36:E36"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="C28:E28"/>
-    <mergeCell ref="C27:E27"/>
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="C34:E34"/>
     <mergeCell ref="C31:E31"/>
@@ -2020,8 +2138,18 @@
     <mergeCell ref="C30:E30"/>
     <mergeCell ref="C21:E21"/>
     <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="C38:E38"/>
+    <mergeCell ref="C32:E32"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="C37:E37"/>
+    <mergeCell ref="C36:E36"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="C27:E27"/>
     <mergeCell ref="C35:E35"/>
-    <mergeCell ref="C25:E25"/>
+    <mergeCell ref="K30:M30"/>
+    <mergeCell ref="K29:M29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>